<commit_message>
Update games tracker with Swing to Secure and Milestone Hopper
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do-Not-Repeat Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -886,103 +886,197 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Archery / angle shooter (Bowman style)</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.crazygames.com/game/bowman</t>
-        </is>
-      </c>
+          <t>Tarzan rope-swing physics traversal (original, rope-swing-style)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Precision coverage against risks</t>
+          <t>Bridging life's gaps - momentum of continuous protection</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Coverage Archer</t>
+          <t>Rope Swing</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Guardian Archer</t>
+          <t>Swing to Secure</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+          <t>Approved - new original concept</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>coverage-archer</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>Revamp</t>
+          <t>swing-to-secure</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Built - Phaser audit pending</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>5037</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Balance runner on a wire</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
-        </is>
-      </c>
+          <t>Crossy Road / Frogger lane-hopping (original, Crossy-Road-style)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Balancing family finances &amp; risks</t>
+          <t>Navigating life's risks to reach each life milestone</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Wire Runner / Balance Dodger</t>
+          <t>Life Crossing</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Tightrope Protection</t>
+          <t>Milestone Hopper</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+          <t>Approved - new original concept</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>milestone-hopper</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>5038</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Archery / angle shooter (Bowman style)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crazygames.com/game/bowman</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Precision coverage against risks</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Archer</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Guardian Archer</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>coverage-archer</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Revamp</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Built - Phaser audit pending</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Balance runner on a wire</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Balancing family finances &amp; risks</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Wire Runner / Balance Dodger</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Tightrope Protection</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
           <t>tightrope-protection</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Revamp</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Built - Phaser audit pending</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K10"/>
+  <autoFilter ref="A1:K12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1020,7 +1114,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
+          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner), swing-to-secure (rope-swing traversal), milestone-hopper (lane-hopper). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register batch-3 games in manifest and regenerate tracker (18 rows)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do-Not-Repeat Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -980,103 +980,432 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Archery / angle shooter (Bowman style)</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.crazygames.com/game/bowman</t>
-        </is>
-      </c>
+          <t>1010! drag-and-place block puzzle (no gravity)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Precision coverage against risks</t>
+          <t>Asset allocation - fitting every asset class into a balanced portfolio</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Coverage Archer</t>
+          <t>Block Fit 1010</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Guardian Archer</t>
+          <t>Portfolio Fit</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+          <t>Ok</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>coverage-archer</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Revamp</t>
+          <t>portfolio-fit</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Built - Phaser audit pending</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
+          <t>Built - review clean (restored)</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>5044</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Balance runner on a wire</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
-        </is>
-      </c>
+          <t>Helix-jump descending ball</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Balancing family finances &amp; risks</t>
+          <t>Riding market cycles - descend through volatility, avoid the crash zones</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Wire Runner / Balance Dodger</t>
+          <t>Helix Descent</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tightrope Protection</t>
+          <t>Spiral Sprint</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+          <t>Approved - new original concept</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>spiral-sprint</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>In Progress (building)</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>5048</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Plinko / pachinko board drop</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Market volatility &amp; ULIP - disciplined investing through ups and downs</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Plinko Pachinko</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Drop</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>wealth-drop</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>In Progress (building)</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>5039</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>One-tap chain reaction</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>One policy protects many - the ripple effect of family coverage</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Chain Reaction</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Ripple Shield</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>ripple-shield</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>In Progress (building)</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>5046</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Jenga-style block removal without toppling</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>De-risking your portfolio without destabilizing your life plan</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Jenga De-Risk</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Steady Tower</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>steady-tower</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>In Progress (building)</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>5047</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Orbit-switch timing arcade</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Staying on track - disciplined orbit around your life goals</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Orbit Hop</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Goal Orbit</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>goal-orbit</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>In Progress (building)</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>5050</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Flick bowling physics</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Knock out risks in one decisive shot - comprehensive cover</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Shield Bowling</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Risk Strike</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>risk-strike</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>In Progress (building)</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>5054</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Archery / angle shooter (Bowman style)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crazygames.com/game/bowman</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Precision coverage against risks</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Archer</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Guardian Archer</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>coverage-archer</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Revamp</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Built - Phaser audit pending</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Balance runner on a wire</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Balancing family finances &amp; risks</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Wire Runner / Balance Dodger</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Tightrope Protection</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
           <t>tightrope-protection</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Revamp</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Built - Phaser audit pending</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K12"/>
+  <autoFilter ref="A1:K19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1114,7 +1443,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner), swing-to-secure (rope-swing traversal), milestone-hopper (lane-hopper). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
+          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner), swing-to-secure (rope-swing traversal), milestone-hopper (lane-hopper), portfolio-fit (1010 block fit — restored after sign-off), spiral-sprint (helix jump), wealth-drop (plinko), ripple-shield (chain reaction), steady-tower (jenga de-risk), goal-orbit (orbit hop), risk-strike (flick bowling). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1455,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Dropped by feedback: Compound Quest (compound-merge), Shield Spin (shield-spin) — 'Already taken'. Removed for lacking BajajLife sign-off: life-goals-bubble-shooter, stackibility-stack, retire-rich-clicker, edurise-jumper, tax-save-maze, she-shield-protector, safe-stride-balancer, portfolio-fit, premium-tiles, income-flow, shield-drop</t>
+          <t>Dropped by feedback: Compound Quest (compound-merge), Shield Spin (shield-spin) — 'Already taken'. Removed for lacking BajajLife sign-off: life-goals-bubble-shooter, stackibility-stack, retire-rich-clicker, edurise-jumper, tax-save-maze, she-shield-protector, safe-stride-balancer, premium-tiles, income-flow, shield-drop. (portfolio-fit was later signed off and restored.)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize tracker: all 16 games built and review clean
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -1064,7 +1064,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>In Progress (building)</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>In Progress (building)</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>In Progress (building)</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>In Progress (building)</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>In Progress (building)</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>In Progress (building)</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">

</xml_diff>

<commit_message>
Register batch 4: manifest, README, kit sync, tracker (28 rows)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es8YGrpPEAvrd8M4hdaYqP
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do-Not-Repeat Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1309,103 +1309,613 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Archery / angle shooter (Bowman style)</t>
+          <t>Pinball flippers (portrait single-screen table)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.crazygames.com/game/bowman</t>
+          <t>Original concept</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Precision coverage against risks</t>
+          <t>Keeping the family's cover in play - every save at the flippers is a premium paid on time</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Coverage Archer</t>
+          <t>Premium Pinball</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Guardian Archer</t>
+          <t>Premium Pinball</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+          <t>Approved - new original concept</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>coverage-archer</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Revamp</t>
+          <t>premium-pinball</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Built - Phaser audit pending</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
+          <t>Built - final fix round in progress</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>5055</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Balance runner on a wire</t>
+          <t>Cricket batting timing (tap-to-swing chase)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+          <t>Original concept</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Balancing family finances &amp; risks</t>
+          <t>Every ball is a life event - cover it with the right timing</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Wire Runner / Balance Dodger</t>
+          <t>Cover Drive</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Tightrope Protection</t>
+          <t>Cover Drive</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+          <t>Approved - new original concept</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>cover-drive</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>5056</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Penalty-save reaction (swipe-to-dive zones)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Cover standing between risk and the family's goals - every save is cover doing its job</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Goal Keeper</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Goal Keeper</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>goal-keeper</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>5057</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Carrom flick-pocket physics (drag striker, pull to aim)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Pocket every goal - the Queen of Protection only stays yours if you cover her</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Carrom</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Carrom</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>wealth-carrom</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>5058</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Press-your-luck inflate (hold to grow, release to bank)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Grow wealth as far as you dare - a Term Shield absorbs the one burst you never saw coming</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Balloon</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Balloon</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>wealth-balloon</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>5059</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Pipe-rotation flow routing puzzle</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Route every rupee of income to the goals that matter - seal the leaks before payday flows</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Income Pipeline</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Income Pipeline</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>income-pipeline</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>5060</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Conveyor swipe-sorting (protect / grow / bin)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Protect it, grow it, or bin it - sort your money life before it scrolls past</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Smart Sorter</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Smart Sorter</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>smart-sorter</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>5061</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Traffic-control tap go/stop (junction management)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Life's traffic never stops - one Claim Cushion, and after that timing is everything</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Safe Crossing</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Safe Crossing</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>safe-crossing</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>5062</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Ice-slide pathing puzzle (swipe, glide to wall)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>One swipe at a time, glide your shield past thin ice and bring it home to the family</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Slide to Safety</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Slide to Safety</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>slide-to-safety</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>5063</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Stop-the-marker precision timing</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pay every premium right on time from 25 to 60 - discipline today is a pension tomorrow</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Perfect Premium</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Perfect Premium</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>perfect-premium</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Built - review clean</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>5064</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Archery / angle shooter (Bowman style)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crazygames.com/game/bowman</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Precision coverage against risks</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Archer</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Guardian Archer</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>coverage-archer</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Revamp</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Built - Phaser audit pending</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Balance runner on a wire</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Balancing family finances &amp; risks</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Wire Runner / Balance Dodger</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Tightrope Protection</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
           <t>tightrope-protection</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>Revamp</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Built - Phaser audit pending</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K19"/>
+  <autoFilter ref="A1:K29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1443,7 +1953,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner), swing-to-secure (rope-swing traversal), milestone-hopper (lane-hopper), portfolio-fit (1010 block fit — restored after sign-off), spiral-sprint (helix jump), wealth-drop (plinko), ripple-shield (chain reaction), steady-tower (jenga de-risk), goal-orbit (orbit hop), risk-strike (flick bowling). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
+          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner), swing-to-secure (rope-swing traversal), milestone-hopper (lane-hopper), portfolio-fit (1010 block fit — restored after sign-off), spiral-sprint (helix jump), wealth-drop (plinko), ripple-shield (chain reaction), steady-tower (jenga de-risk), goal-orbit (orbit hop), risk-strike (flick bowling), premium-pinball (pinball flippers), cover-drive (cricket batting timing), goal-keeper (penalty-save reaction), wealth-carrom (carrom flick-pocket), wealth-balloon (press-your-luck inflate), income-pipeline (pipe-rotation flow routing), smart-sorter (conveyor swipe-sorting), safe-crossing (traffic-control tap go/stop), slide-to-safety (ice-slide pathing), perfect-premium (stop-the-marker precision). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track batch 5 in tracker: 5 arcade games in build (33 rows)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es8YGrpPEAvrd8M4hdaYqP
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do-Not-Repeat Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1819,103 +1819,358 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Archery / angle shooter (Bowman style)</t>
+          <t>One-tap impulse flight through gates (flappy-style)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>https://www.crazygames.com/game/bowman</t>
+          <t>Original concept</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Precision coverage against risks</t>
+          <t>Life's expenses keep coming - keep your cover airborne and glide through every one</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Coverage Archer</t>
+          <t>Steady Wings</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Guardian Archer</t>
+          <t>Steady Wings</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+          <t>Approved - new original concept</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>coverage-archer</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Revamp</t>
+          <t>steady-wings</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Built - Phaser audit pending</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
+          <t>In build - agent running</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>5065</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Balance runner on a wire</t>
+          <t>Beat-synchronised rhythm tapping (radial go/no-go)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+          <t>Original concept</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Balancing family finances &amp; risks</t>
+          <t>A premium on every beat - stay in rhythm, skip the temptations, and cover never misses</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Wire Runner / Balance Dodger</t>
+          <t>Premium Pulse</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Tightrope Protection</t>
+          <t>Premium Pulse</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+          <t>Approved - new original concept</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
+          <t>premium-pulse</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>In build - agent running</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>5066</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Simon-style serial sequence recall (ordered memory)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>A financial plan only works if you remember every step - recall it in order, skip the risky detours</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Smart Recall</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Smart Recall</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>smart-recall</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>In build - agent running</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>5067</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Tap-to-bounce juggling keep-ups (multi-body physics)</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Real life means keeping every goal in the air at once - cover is what catches the one you miss</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Goal Juggler</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Goal Juggler</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>goal-juggler</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>In build - agent running</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>5068</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>WarioWare-style microgame rush (3-5s one-verb challenges)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Original concept</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Life comes at you fast - pay, protect, pick and plan in seconds; that is what good cover feels like</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Life Rush</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Life Rush</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Approved - new original concept</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>life-rush</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>In build - agent running</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>5069</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Archery / angle shooter (Bowman style)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crazygames.com/game/bowman</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Precision coverage against risks</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Archer</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Guardian Archer</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>coverage-archer</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Revamp</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Built - Phaser audit pending</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Balance runner on a wire</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Balancing family finances &amp; risks</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Wire Runner / Balance Dodger</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Tightrope Protection</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
           <t>tightrope-protection</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>Revamp</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Built - Phaser audit pending</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K29"/>
+  <autoFilter ref="A1:K34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Premium-pulse review clean; tracker status update
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es8YGrpPEAvrd8M4hdaYqP
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -1350,7 +1350,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Built - final fix round in progress</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>In build - agent running</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>In build - agent running</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>In build - agent running</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">

</xml_diff>

<commit_message>
Register batch 5: README, kit sync, catalog note, tracker at 33 games
Goal-juggler and life-rush flip to review clean; steady-wings,
premium-pulse, smart-recall, goal-juggler, life-rush added to the games
table (5065-5069), the kit sync list and the approved-scope catalog
note. GAMES_TRACKER.xlsx regenerated: 33 rows, all built games review
clean.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es8YGrpPEAvrd8M4hdaYqP
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -2013,7 +2013,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>In build - agent running</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K31" s="2" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>In build - agent running</t>
+          <t>Built - review clean</t>
         </is>
       </c>
       <c r="K32" s="2" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner), swing-to-secure (rope-swing traversal), milestone-hopper (lane-hopper), portfolio-fit (1010 block fit — restored after sign-off), spiral-sprint (helix jump), wealth-drop (plinko), ripple-shield (chain reaction), steady-tower (jenga de-risk), goal-orbit (orbit hop), risk-strike (flick bowling), premium-pinball (pinball flippers), cover-drive (cricket batting timing), goal-keeper (penalty-save reaction), wealth-carrom (carrom flick-pocket), wealth-balloon (press-your-luck inflate), income-pipeline (pipe-rotation flow routing), smart-sorter (conveyor swipe-sorting), safe-crossing (traffic-control tap go/stop), slide-to-safety (ice-slide pathing), perfect-premium (stop-the-marker precision). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
+          <t>guardian-shelter (shield physics), secure-journey (rail shooter), smart-match-3d (triple match), risk-exit (arrow puzzle), life-soar (glider), coverage-archer (archery), tightrope-protection (balance runner), swing-to-secure (rope-swing traversal), milestone-hopper (lane-hopper), portfolio-fit (1010 block fit — restored after sign-off), spiral-sprint (helix jump), wealth-drop (plinko), ripple-shield (chain reaction), steady-tower (jenga de-risk), goal-orbit (orbit hop), risk-strike (flick bowling), premium-pinball (pinball flippers), cover-drive (cricket batting timing), goal-keeper (penalty-save reaction), wealth-carrom (carrom flick-pocket), wealth-balloon (press-your-luck inflate), income-pipeline (pipe-rotation flow routing), smart-sorter (conveyor swipe-sorting), safe-crossing (traffic-control tap go/stop), slide-to-safety (ice-slide pathing), perfect-premium (stop-the-marker precision), steady-wings (one-tap impulse flight), premium-pulse (beat-synced rhythm tapping), smart-recall (Simon serial sequence recall), goal-juggler (tap-to-bounce juggling keep-ups), life-rush (rapid-fire microgame rush). Approved but not yet scaffolded: balance-block-journey, shield-cascade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register batch 6: README, kit sync, catalog note, tracker at 38 rows
Five viral-genre proposals pending BajajLife sign-off: guardian-arena,
premium-tiles, wealth-merge, risk-slash, sip-stack (ports 5070-5074).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do-Not-Repeat Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2074,103 +2074,358 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Archery / angle shooter (Bowman style)</t>
+          <t>Archero-style arena survivor (stop-to-shoot, wave upgrades)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>https://www.crazygames.com/game/bowman</t>
+          <t>https://apps.apple.com/app/archero/id1453651052</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Precision coverage against risks</t>
+          <t>Layered protection - every upgrade between waves is another rider on the family's cover</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Coverage Archer</t>
+          <t>Guardian Arena</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Guardian Archer</t>
+          <t>Guardian Arena</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+          <t>Proposed 2026-07-29 - pending BajajLife sign-off</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>coverage-archer</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>Revamp</t>
+          <t>guardian-arena</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Built - Phaser audit pending</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr"/>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>5070</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Balance runner on a wire</t>
+          <t>Piano Tiles-style 4-lane melody tapper</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+          <t>https://apps.apple.com/app/piano-tiles-2/id1027688889</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Balancing family finances &amp; risks</t>
+          <t>A premium on every note - never miss a payment and the family's plan plays like music</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Wire Runner / Balance Dodger</t>
+          <t>Premium Tiles</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Tightrope Protection</t>
+          <t>Premium Tiles</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+          <t>Proposed 2026-07-29 - pending BajajLife sign-off. Note: an earlier premium-tiles concept was removed in the 2026-07-28 scope cut for lacking sign-off; this is a fresh implementation of the explicitly requested piano-tiles genre</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
+          <t>premium-tiles</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>5071</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Suika-style drop-and-merge collector (physics jar)</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/app/suika-game-aladdin-x/id6444114954</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Compounding in your hands - small savings merge into life goals</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Merge</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Merge</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Proposed 2026-07-29 - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>wealth-merge</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>5072</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Fruit Ninja-style swipe slicer (slash risks, spare shields)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/app/fruit-ninja/id362949845</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Cut the risks out of the family's life - cover is the blade</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Risk Slash</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Risk Slash</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Proposed 2026-07-29 - pending BajajLife sign-off. Note: bajaj-game-store catalog lists a fruit-slice game; this differentiates via the protect-the-Family-Shield rule (slicing blue shield orbs is the penalty) and risk-labelled targets</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>risk-slash</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>5073</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Ketchapp Stack-style timing tower (trim on miss, regrow on perfects)</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/app/stack/id1080487957</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Every layer is a monthly SIP - discipline compounds, and consistency repairs old mistakes</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>SIP Stack</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>SIP Stack</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Proposed 2026-07-29 - pending BajajLife sign-off. Note: bajaj-game-store catalog lists a stacking game; this differentiates via SIP milestone framing and the perfect-streak width-regrowth loop</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>sip-stack</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>5074</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Archery / angle shooter (Bowman style)</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crazygames.com/game/bowman</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Precision coverage against risks</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Archer</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Guardian Archer</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>coverage-archer</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Revamp</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Built - Phaser audit pending</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Balance runner on a wire</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Balancing family finances &amp; risks</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Wire Runner / Balance Dodger</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Tightrope Protection</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
           <t>tightrope-protection</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>Revamp</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>Built - Phaser audit pending</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K34"/>
+  <autoFilter ref="A1:K39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2181,7 +2436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2215,34 +2470,46 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Removed from repo</t>
+          <t>This repo (proposed, pending sign-off)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Dropped by feedback: Compound Quest (compound-merge), Shield Spin (shield-spin) — 'Already taken'. Removed for lacking BajajLife sign-off: life-goals-bubble-shooter, stackibility-stack, retire-rich-clicker, edurise-jumper, tax-save-maze, she-shield-protector, safe-stride-balancer, premium-tiles, income-flow, shield-drop. (portfolio-fit was later signed off and restored.)</t>
+          <t>Batch 6 (2026-07-29): guardian-arena (Archero-style arena survivor), premium-tiles (piano-tiles melody lane tapper), wealth-merge (suika drop-merge collector), risk-slash (swipe slicer with protect-the-shield rule; note game-store has fruit-slice), sip-stack (stack timing tower with SIP framing; note game-store has stacking)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>bajaj-game-store (do not repeat)</t>
+          <t>Removed from repo</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>snake, hangman, word scramble, match-3 x2, tetris, fruit-slice, runners/climbers x4, top-down shooter, bomberman, galaga, sudoku x2, whack-a-mole x2, brick-breaker, jigsaw x2, minesweeper, racing, tube-sorting, quiz x3, bubble shooter, peg solitaire, stacking, memory-flip, tower defense, snakes &amp; ladders, arcade dodger</t>
+          <t>Dropped by feedback: Compound Quest (compound-merge), Shield Spin (shield-spin) — 'Already taken'. Removed for lacking BajajLife sign-off: life-goals-bubble-shooter, stackibility-stack, retire-rich-clicker, edurise-jumper, tax-save-maze, she-shield-protector, safe-stride-balancer, premium-tiles, income-flow, shield-drop. (portfolio-fit was later signed off and restored.)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>bajaj-game-store (do not repeat)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>snake, hangman, word scramble, match-3 x2, tetris, fruit-slice, runners/climbers x4, top-down shooter, bomberman, galaga, sudoku x2, whack-a-mole x2, brick-breaker, jigsaw x2, minesweeper, racing, tube-sorting, quiz x3, bubble shooter, peg solitaire, stacking, memory-flip, tower defense, snakes &amp; ladders, arcade dodger</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>Dropped by feedback</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Wealth Current (physics orb), Path to Legacy (line drawing), Launch to Protection (hedgehog launch), Secure Foundations (falling sand)</t>
         </is>

</xml_diff>

<commit_message>
Register batch 7: README, kit sync, catalog note, tracker at 43 rows
Five rare-mechanic proposals pending BajajLife sign-off: legacy-echo,
time-shield, ring-fence, risk-radar, dual-cover (ports 5075-5079), each
with a headless gate.mjs fairness/solvability proof.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GAMES_TRACKER.xlsx
+++ b/GAMES_TRACKER.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do-Not-Repeat Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games Tracker'!$A$1:$K$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2329,103 +2329,338 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Archery / angle shooter (Bowman style)</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.crazygames.com/game/bowman</t>
-        </is>
-      </c>
+          <t>Time-loop past-self co-op (previous runs replay as live ghost helpers)</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Precision coverage against risks</t>
+          <t>Your past contributions keep working for you - every premium your past self paid protects the family today</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Coverage Archer</t>
+          <t>Legacy Echo</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Guardian Archer</t>
+          <t>Legacy Echo</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+          <t>Proposed 2026-07-30 - pending BajajLife sign-off</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>coverage-archer</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>Revamp</t>
+          <t>legacy-echo</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Built - Phaser audit pending</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr"/>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>5075</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Balance runner on a wire</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
-        </is>
-      </c>
+          <t>Time moves only when you move (SUPERHOT rule)</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Balancing family finances &amp; risks</t>
+          <t>Good cover buys you time to think - slow life down and pick your path</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Wire Runner / Balance Dodger</t>
+          <t>Time Shield</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Tightrope Protection</t>
+          <t>Time Shield</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+          <t>Proposed 2026-07-30 - pending BajajLife sign-off</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
+          <t>time-shield</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>5076</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Qix/JezzBall territory capture (claim ground, wall risks out)</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Ring-fence the family's wealth - a real asset-protection term made playable</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Ring-Fence</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Ring-Fence</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Proposed 2026-07-30 - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>ring-fence</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>5077</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Darkness + sonar pulse navigation (perception as a resource)</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>You cannot see risks coming - your cover can; send the radar, read the danger, walk the family home</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Risk Radar</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Risk Radar</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Proposed 2026-07-30 - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>risk-radar</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>5078</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Duet-style twin-orbit dodger (one input, two coupled avatars)</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Protection and growth are two sides of one plan - steer them together; losing either loses the future</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Dual Cover</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Dual Cover</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Proposed 2026-07-30 - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>dual-cover</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Built - pending BajajLife sign-off</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>5079</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Archery / angle shooter (Bowman style)</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crazygames.com/game/bowman</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Precision coverage against risks</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Archer</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Guardian Archer</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Make single player: replace the other human opponent with virus targets; ONLY our player can fire (no return fire)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>coverage-archer</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Revamp</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Built - Phaser audit pending</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Balance runner on a wire</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.miniplay.com/game/bug-on-a-wire</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Balancing family finances &amp; risks</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Wire Runner / Balance Dodger</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Tightrope Protection</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Ok, Replace crows with risks {Risk = Green virus} Remove wire, it must be on flat ground.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
           <t>tightrope-protection</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Revamp</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Built - Phaser audit pending</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K39"/>
+  <autoFilter ref="A1:K44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2475,7 +2710,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Batch 6 (2026-07-29): guardian-arena (Archero-style arena survivor), premium-tiles (piano-tiles melody lane tapper), wealth-merge (suika drop-merge collector), risk-slash (swipe slicer with protect-the-shield rule; note game-store has fruit-slice), sip-stack (stack timing tower with SIP framing; note game-store has stacking)</t>
+          <t>Batch 6 (2026-07-29): guardian-arena (Archero-style arena survivor), premium-tiles (piano-tiles melody lane tapper), wealth-merge (suika drop-merge collector), risk-slash (swipe slicer with protect-the-shield rule; note game-store has fruit-slice), sip-stack (stack timing tower with SIP framing; note game-store has stacking). Batch 7 (2026-07-30): legacy-echo (time-loop past-self co-op), time-shield (time moves only when you move), ring-fence (Qix territory capture), risk-radar (darkness + sonar pulse navigation), dual-cover (Duet twin-orbit dodger)</t>
         </is>
       </c>
     </row>

</xml_diff>